<commit_message>
Name all header columns (E-M) on Main sheet
Replace letter placeholders (C-K) with descriptive header names:
E=Selected Vacancy URL, F=Deputation Vacancy URL,
G=Deputation Page (Same/Separate), H=Deputation Vacancies Available (Yes/No),
I=Confidence Level, J=Remarks, K=Last Verified Date,
L=Dedicated Recruitment Portal (Yes/No), M=Source Type.
H and L names are inferred (were undefined) pending confirmation.
</commit_message>
<xml_diff>
--- a/Master list - Ministries and Departments.xlsx
+++ b/Master list - Ministries and Departments.xlsx
@@ -17,10 +17,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="dd-mm-yyyy"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -432,49 +431,49 @@
           <t>Organisation Type</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>E</t>
-        </is>
-      </c>
-      <c r="H1" s="2" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="I1" s="2" t="inlineStr">
-        <is>
-          <t>G</t>
-        </is>
-      </c>
-      <c r="J1" s="2" t="inlineStr">
-        <is>
-          <t>H</t>
-        </is>
-      </c>
-      <c r="K1" s="2" t="inlineStr">
-        <is>
-          <t>I</t>
-        </is>
-      </c>
-      <c r="L1" s="2" t="inlineStr">
-        <is>
-          <t>J</t>
-        </is>
-      </c>
-      <c r="M1" s="2" t="inlineStr">
-        <is>
-          <t>K</t>
+      <c r="E1" s="4" t="inlineStr">
+        <is>
+          <t>Selected Vacancy URL</t>
+        </is>
+      </c>
+      <c r="F1" s="4" t="inlineStr">
+        <is>
+          <t>Deputation Vacancy URL</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Deputation Page (Same / Separate)</t>
+        </is>
+      </c>
+      <c r="H1" s="4" t="inlineStr">
+        <is>
+          <t>Deputation Vacancies Available (Yes/No)</t>
+        </is>
+      </c>
+      <c r="I1" s="4" t="inlineStr">
+        <is>
+          <t>Confidence Level</t>
+        </is>
+      </c>
+      <c r="J1" s="4" t="inlineStr">
+        <is>
+          <t>Remarks</t>
+        </is>
+      </c>
+      <c r="K1" s="4" t="inlineStr">
+        <is>
+          <t>Last Verified Date</t>
+        </is>
+      </c>
+      <c r="L1" s="4" t="inlineStr">
+        <is>
+          <t>Dedicated Recruitment Portal (Yes/No)</t>
+        </is>
+      </c>
+      <c r="M1" s="4" t="inlineStr">
+        <is>
+          <t>Source Type</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refine headers per clarification: E=vacancy/recruitment ad page URL, G=deputation page same as vacancy page (Yes/No)
- Rename E header to 'Vacancy / Recruitment Advertisement Page URL'.
- Rename G header to 'Deputation Page Same as Vacancy Page' and convert
  values from Same Page/Separate Page to Yes/No (Yes=same as vacancy page).
- F (Deputation Vacancy URL) holds the separate URL only when G=No (~5% of cases).
</commit_message>
<xml_diff>
--- a/Master list - Ministries and Departments.xlsx
+++ b/Master list - Ministries and Departments.xlsx
@@ -433,7 +433,7 @@
       </c>
       <c r="E1" s="4" t="inlineStr">
         <is>
-          <t>Selected Vacancy URL</t>
+          <t>Vacancy / Recruitment Advertisement Page URL</t>
         </is>
       </c>
       <c r="F1" s="4" t="inlineStr">
@@ -443,7 +443,7 @@
       </c>
       <c r="G1" s="4" t="inlineStr">
         <is>
-          <t>Deputation Page (Same / Separate)</t>
+          <t>Deputation Page Same as Vacancy Page</t>
         </is>
       </c>
       <c r="H1" s="4" t="inlineStr">
@@ -539,7 +539,7 @@
       </c>
       <c r="G3" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H3" s="11" t="inlineStr">
@@ -603,7 +603,7 @@
       </c>
       <c r="G4" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H4" s="11" t="inlineStr">
@@ -667,7 +667,7 @@
       </c>
       <c r="G5" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H5" s="11" t="inlineStr">
@@ -731,7 +731,7 @@
       </c>
       <c r="G6" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H6" s="11" t="inlineStr">
@@ -795,7 +795,7 @@
       </c>
       <c r="G7" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H7" s="11" t="inlineStr">
@@ -859,7 +859,7 @@
       </c>
       <c r="G8" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H8" s="11" t="inlineStr">
@@ -923,7 +923,7 @@
       </c>
       <c r="G9" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H9" s="11" t="inlineStr">
@@ -987,7 +987,7 @@
       </c>
       <c r="G10" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H10" s="11" t="inlineStr">
@@ -1081,7 +1081,7 @@
       </c>
       <c r="G12" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H12" s="11" t="inlineStr">
@@ -1145,7 +1145,7 @@
       </c>
       <c r="G13" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H13" s="11" t="inlineStr">
@@ -1209,7 +1209,7 @@
       </c>
       <c r="G14" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H14" s="11" t="inlineStr">
@@ -1273,7 +1273,7 @@
       </c>
       <c r="G15" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H15" s="11" t="inlineStr">
@@ -1337,7 +1337,7 @@
       </c>
       <c r="G16" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H16" s="11" t="inlineStr">
@@ -1401,7 +1401,7 @@
       </c>
       <c r="G17" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H17" s="11" t="inlineStr">
@@ -1465,7 +1465,7 @@
       </c>
       <c r="G18" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H18" s="11" t="inlineStr">
@@ -1529,7 +1529,7 @@
       </c>
       <c r="G19" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H19" s="11" t="inlineStr">
@@ -1593,7 +1593,7 @@
       </c>
       <c r="G20" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H20" s="11" t="inlineStr">
@@ -1657,7 +1657,7 @@
       </c>
       <c r="G21" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H21" s="11" t="inlineStr">
@@ -1721,7 +1721,7 @@
       </c>
       <c r="G22" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H22" s="11" t="inlineStr">
@@ -1785,7 +1785,7 @@
       </c>
       <c r="G23" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H23" s="11" t="inlineStr">
@@ -1849,7 +1849,7 @@
       </c>
       <c r="G24" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H24" s="11" t="inlineStr">
@@ -1913,7 +1913,7 @@
       </c>
       <c r="G25" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H25" s="11" t="inlineStr">
@@ -2007,7 +2007,7 @@
       </c>
       <c r="G27" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H27" s="11" t="inlineStr">
@@ -2071,7 +2071,7 @@
       </c>
       <c r="G28" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H28" s="11" t="inlineStr">
@@ -2135,7 +2135,7 @@
       </c>
       <c r="G29" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H29" s="11" t="inlineStr">
@@ -2199,7 +2199,7 @@
       </c>
       <c r="G30" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H30" s="11" t="inlineStr">
@@ -2263,7 +2263,7 @@
       </c>
       <c r="G31" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H31" s="11" t="inlineStr">
@@ -2327,7 +2327,7 @@
       </c>
       <c r="G32" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H32" s="11" t="inlineStr">
@@ -2391,7 +2391,7 @@
       </c>
       <c r="G33" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H33" s="11" t="inlineStr">
@@ -2455,7 +2455,7 @@
       </c>
       <c r="G34" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H34" s="11" t="inlineStr">
@@ -18176,7 +18176,7 @@
       </c>
       <c r="G553" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H553" s="11" t="inlineStr">
@@ -18240,7 +18240,7 @@
       </c>
       <c r="G554" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H554" s="11" t="inlineStr">
@@ -18304,7 +18304,7 @@
       </c>
       <c r="G555" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H555" s="11" t="inlineStr">
@@ -18368,7 +18368,7 @@
       </c>
       <c r="G556" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H556" s="11" t="inlineStr">
@@ -18432,7 +18432,7 @@
       </c>
       <c r="G557" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H557" s="11" t="inlineStr">
@@ -18496,7 +18496,7 @@
       </c>
       <c r="G558" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H558" s="11" t="inlineStr">
@@ -18560,7 +18560,7 @@
       </c>
       <c r="G559" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H559" s="11" t="inlineStr">
@@ -18624,7 +18624,7 @@
       </c>
       <c r="G560" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H560" s="11" t="inlineStr">
@@ -18688,7 +18688,7 @@
       </c>
       <c r="G561" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H561" s="11" t="inlineStr">
@@ -18752,7 +18752,7 @@
       </c>
       <c r="G562" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H562" s="11" t="inlineStr">
@@ -18846,7 +18846,7 @@
       </c>
       <c r="G564" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H564" s="11" t="inlineStr">
@@ -18910,7 +18910,7 @@
       </c>
       <c r="G565" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H565" s="11" t="inlineStr">
@@ -18974,7 +18974,7 @@
       </c>
       <c r="G566" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H566" s="11" t="inlineStr">
@@ -19038,7 +19038,7 @@
       </c>
       <c r="G567" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H567" s="11" t="inlineStr">
@@ -19102,7 +19102,7 @@
       </c>
       <c r="G568" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H568" s="11" t="inlineStr">
@@ -19166,7 +19166,7 @@
       </c>
       <c r="G569" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H569" s="11" t="inlineStr">
@@ -19230,7 +19230,7 @@
       </c>
       <c r="G570" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H570" s="11" t="inlineStr">
@@ -19294,7 +19294,7 @@
       </c>
       <c r="G571" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H571" s="11" t="inlineStr">
@@ -19358,7 +19358,7 @@
       </c>
       <c r="G572" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H572" s="11" t="inlineStr">
@@ -19422,7 +19422,7 @@
       </c>
       <c r="G573" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H573" s="11" t="inlineStr">
@@ -19486,7 +19486,7 @@
       </c>
       <c r="G574" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H574" s="11" t="inlineStr">
@@ -19550,7 +19550,7 @@
       </c>
       <c r="G575" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H575" s="11" t="inlineStr">
@@ -19644,7 +19644,7 @@
       </c>
       <c r="G577" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H577" s="11" t="inlineStr">
@@ -19708,7 +19708,7 @@
       </c>
       <c r="G578" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H578" s="11" t="inlineStr">
@@ -19772,7 +19772,7 @@
       </c>
       <c r="G579" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H579" s="11" t="inlineStr">
@@ -19836,7 +19836,7 @@
       </c>
       <c r="G580" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H580" s="11" t="inlineStr">
@@ -19900,7 +19900,7 @@
       </c>
       <c r="G581" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H581" s="11" t="inlineStr">
@@ -19964,7 +19964,7 @@
       </c>
       <c r="G582" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H582" s="11" t="inlineStr">
@@ -20028,7 +20028,7 @@
       </c>
       <c r="G583" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H583" s="11" t="inlineStr">
@@ -20092,7 +20092,7 @@
       </c>
       <c r="G584" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H584" s="11" t="inlineStr">
@@ -20156,7 +20156,7 @@
       </c>
       <c r="G585" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H585" s="11" t="inlineStr">
@@ -20220,7 +20220,7 @@
       </c>
       <c r="G586" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H586" s="11" t="inlineStr">
@@ -20314,7 +20314,7 @@
       </c>
       <c r="G588" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H588" s="11" t="inlineStr">
@@ -20378,7 +20378,7 @@
       </c>
       <c r="G589" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H589" s="11" t="inlineStr">
@@ -20442,7 +20442,7 @@
       </c>
       <c r="G590" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H590" s="11" t="inlineStr">
@@ -20506,7 +20506,7 @@
       </c>
       <c r="G591" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H591" s="11" t="inlineStr">
@@ -20570,7 +20570,7 @@
       </c>
       <c r="G592" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H592" s="11" t="inlineStr">
@@ -20634,7 +20634,7 @@
       </c>
       <c r="G593" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H593" s="11" t="inlineStr">
@@ -20698,7 +20698,7 @@
       </c>
       <c r="G594" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H594" s="11" t="inlineStr">
@@ -20762,7 +20762,7 @@
       </c>
       <c r="G595" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H595" s="11" t="inlineStr">
@@ -20856,7 +20856,7 @@
       </c>
       <c r="G597" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H597" s="11" t="inlineStr">
@@ -20920,7 +20920,7 @@
       </c>
       <c r="G598" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H598" s="11" t="inlineStr">
@@ -20984,7 +20984,7 @@
       </c>
       <c r="G599" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H599" s="11" t="inlineStr">
@@ -21048,7 +21048,7 @@
       </c>
       <c r="G600" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H600" s="11" t="inlineStr">
@@ -21112,7 +21112,7 @@
       </c>
       <c r="G601" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H601" s="11" t="inlineStr">
@@ -21176,7 +21176,7 @@
       </c>
       <c r="G602" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H602" s="11" t="inlineStr">
@@ -21270,7 +21270,7 @@
       </c>
       <c r="G604" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H604" s="11" t="inlineStr">
@@ -21334,7 +21334,7 @@
       </c>
       <c r="G605" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H605" s="11" t="inlineStr">
@@ -21398,7 +21398,7 @@
       </c>
       <c r="G606" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H606" s="11" t="inlineStr">
@@ -21462,7 +21462,7 @@
       </c>
       <c r="G607" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H607" s="11" t="inlineStr">
@@ -21526,7 +21526,7 @@
       </c>
       <c r="G608" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H608" s="11" t="inlineStr">
@@ -21590,7 +21590,7 @@
       </c>
       <c r="G609" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H609" s="11" t="inlineStr">
@@ -21654,7 +21654,7 @@
       </c>
       <c r="G610" s="11" t="inlineStr">
         <is>
-          <t>Same Page</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H610" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Batch 1/3: replace 10 homepage URLs with deep recruitment links
AYUSH bodies -> central recruitment portal / own recruitment pages:
R13 AIIA, R15 NIUM, R20 CCRS, R21 CCRH, R22 CCRYN -> recruitment.ayush.gov.in
R17 NIH -> nih.ayush.gov.in/recruitment (domain migrated from nih.nic.in)
R23 NCISM -> ncismindia.org/advertisements.php
R25 PCIM&H -> pcimh.gov.in/index.php/recruitment
R556 EMRS -> emrs.tribal.gov.in (dedicated recruitment portal)
R33 PCI -> domain corrected to pci.gov.in (SPA; flagged Low, needs manual check)
</commit_message>
<xml_diff>
--- a/Master list - Ministries and Departments.xlsx
+++ b/Master list - Ministries and Departments.xlsx
@@ -1031,12 +1031,12 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>https://aiia.gov.in/</t>
+          <t>https://recruitment.ayush.gov.in/</t>
         </is>
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>https://aiia.gov.in/</t>
+          <t>https://recruitment.ayush.gov.in/</t>
         </is>
       </c>
       <c r="G13" s="11" t="inlineStr">
@@ -1046,12 +1046,12 @@
       </c>
       <c r="H13" s="11" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I13" s="11" t="inlineStr">
         <is>
-          <t>AIIA posts recruitment notices on its official site; stable deep recruitment URL not confirmed.</t>
+          <t>AYUSH central recruitment portal (covers AIIA); AIIA also runs aiiarecruitment.org. Replaces homepage.</t>
         </is>
       </c>
       <c r="J13" s="17" t="n">
@@ -1059,7 +1059,7 @@
       </c>
       <c r="K13" s="11" t="inlineStr">
         <is>
-          <t>Website</t>
+          <t>Portal</t>
         </is>
       </c>
     </row>
@@ -1139,12 +1139,12 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>https://www.nium.in/</t>
+          <t>https://recruitment.ayush.gov.in/</t>
         </is>
       </c>
       <c r="F15" s="6" t="inlineStr">
         <is>
-          <t>https://www.nium.in/</t>
+          <t>https://recruitment.ayush.gov.in/</t>
         </is>
       </c>
       <c r="G15" s="11" t="inlineStr">
@@ -1154,12 +1154,12 @@
       </c>
       <c r="H15" s="11" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I15" s="11" t="inlineStr">
         <is>
-          <t>NIUM recruitment notices on official site; dedicated page not auto-confirmed.</t>
+          <t>AYUSH central recruitment portal lists NIUM. Replaces homepage.</t>
         </is>
       </c>
       <c r="J15" s="17" t="n">
@@ -1167,7 +1167,7 @@
       </c>
       <c r="K15" s="11" t="inlineStr">
         <is>
-          <t>Website</t>
+          <t>Portal</t>
         </is>
       </c>
     </row>
@@ -1247,12 +1247,12 @@
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>https://www.nih.nic.in/</t>
+          <t>https://www.nih.ayush.gov.in/recruitment</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>https://www.nih.nic.in/</t>
+          <t>https://www.nih.ayush.gov.in/recruitment</t>
         </is>
       </c>
       <c r="G17" s="11" t="inlineStr">
@@ -1262,12 +1262,12 @@
       </c>
       <c r="H17" s="11" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I17" s="11" t="inlineStr">
         <is>
-          <t>NIH Kolkata recruitment notices on official site; dedicated page not auto-confirmed.</t>
+          <t>NIH recruitment page; domain migrated nih.nic.in -&gt; nih.ayush.gov.in. Replaces homepage.</t>
         </is>
       </c>
       <c r="J17" s="17" t="n">
@@ -1409,12 +1409,12 @@
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>https://ccrsindia.res.in/</t>
+          <t>https://recruitment.ayush.gov.in/</t>
         </is>
       </c>
       <c r="F20" s="6" t="inlineStr">
         <is>
-          <t>https://ccrsindia.res.in/</t>
+          <t>https://recruitment.ayush.gov.in/</t>
         </is>
       </c>
       <c r="G20" s="11" t="inlineStr">
@@ -1424,12 +1424,12 @@
       </c>
       <c r="H20" s="11" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I20" s="11" t="inlineStr">
         <is>
-          <t>Official CCRS domain; site not reachable for deep-link confirmation from here.</t>
+          <t>AYUSH central recruitment portal lists CCRS; walk-ins also on ccrs.ayush.gov.in. Replaces homepage.</t>
         </is>
       </c>
       <c r="J20" s="17" t="n">
@@ -1437,7 +1437,7 @@
       </c>
       <c r="K20" s="11" t="inlineStr">
         <is>
-          <t>Website</t>
+          <t>Portal</t>
         </is>
       </c>
     </row>
@@ -1463,12 +1463,12 @@
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>https://www.ccrhindia.nic.in/</t>
+          <t>https://recruitment.ayush.gov.in/</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>https://www.ccrhindia.nic.in/</t>
+          <t>https://recruitment.ayush.gov.in/</t>
         </is>
       </c>
       <c r="G21" s="11" t="inlineStr">
@@ -1483,7 +1483,7 @@
       </c>
       <c r="I21" s="11" t="inlineStr">
         <is>
-          <t>Official CCRH domain; deep recruitment link not auto-confirmed.</t>
+          <t>AYUSH central recruitment portal; CCRH also advertises on its own AYUSH site. Replaces homepage.</t>
         </is>
       </c>
       <c r="J21" s="17" t="n">
@@ -1491,7 +1491,7 @@
       </c>
       <c r="K21" s="11" t="inlineStr">
         <is>
-          <t>Website</t>
+          <t>Portal</t>
         </is>
       </c>
     </row>
@@ -1517,12 +1517,12 @@
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>https://ccryn.gov.in/</t>
+          <t>https://recruitment.ayush.gov.in/</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
         <is>
-          <t>https://ccryn.gov.in/</t>
+          <t>https://recruitment.ayush.gov.in/</t>
         </is>
       </c>
       <c r="G22" s="11" t="inlineStr">
@@ -1537,7 +1537,7 @@
       </c>
       <c r="I22" s="11" t="inlineStr">
         <is>
-          <t>Official CCRYN domain; deep recruitment link not auto-confirmed.</t>
+          <t>AYUSH central recruitment portal; CCRYN also advertises on ccryn.gov.in. Replaces homepage.</t>
         </is>
       </c>
       <c r="J22" s="17" t="n">
@@ -1545,7 +1545,7 @@
       </c>
       <c r="K22" s="11" t="inlineStr">
         <is>
-          <t>Website</t>
+          <t>Portal</t>
         </is>
       </c>
     </row>
@@ -1571,12 +1571,12 @@
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>https://ncismindia.org/</t>
+          <t>https://www.ncismindia.org/advertisements.php</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>https://ncismindia.org/</t>
+          <t>https://www.ncismindia.org/advertisements.php</t>
         </is>
       </c>
       <c r="G23" s="11" t="inlineStr">
@@ -1586,12 +1586,12 @@
       </c>
       <c r="H23" s="11" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I23" s="11" t="inlineStr">
         <is>
-          <t>CCIM superseded by NCISM (National Commission for Indian System of Medicine); link points to NCISM.</t>
+          <t>NCISM recruitment advertisements page (replaces homepage).</t>
         </is>
       </c>
       <c r="J23" s="17" t="n">
@@ -1679,12 +1679,12 @@
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>https://pcimh.gov.in/</t>
+          <t>https://pcimh.gov.in/index.php/recruitment</t>
         </is>
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>https://pcimh.gov.in/</t>
+          <t>https://pcimh.gov.in/index.php/recruitment</t>
         </is>
       </c>
       <c r="G25" s="11" t="inlineStr">
@@ -1694,12 +1694,12 @@
       </c>
       <c r="H25" s="11" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I25" s="11" t="inlineStr">
         <is>
-          <t>PCIM&amp;H official site; dedicated recruitment page not auto-confirmed.</t>
+          <t>PCIM&amp;H recruitment page (replaces homepage).</t>
         </is>
       </c>
       <c r="J25" s="17" t="n">
@@ -2085,12 +2085,12 @@
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>https://www.pci.nic.in/</t>
+          <t>https://www.pci.gov.in/</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr">
         <is>
-          <t>https://www.pci.nic.in/</t>
+          <t>https://www.pci.gov.in/</t>
         </is>
       </c>
       <c r="G33" s="11" t="inlineStr">
@@ -2100,12 +2100,12 @@
       </c>
       <c r="H33" s="11" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I33" s="11" t="inlineStr">
         <is>
-          <t>Pharmacy Council of India official site; deep recruitment link not auto-confirmed.</t>
+          <t>Domain corrected pci.nic.in -&gt; pci.gov.in. Site is a SPA exposing no stable recruitment-route URL; vacancy notices appear within portal. NEEDS MANUAL CONFIRMATION.</t>
         </is>
       </c>
       <c r="J33" s="17" t="n">
@@ -16976,12 +16976,12 @@
       </c>
       <c r="E556" s="11" t="inlineStr">
         <is>
-          <t>https://nests.tribal.gov.in/</t>
+          <t>https://www.emrs.tribal.gov.in/</t>
         </is>
       </c>
       <c r="F556" s="11" t="inlineStr">
         <is>
-          <t>https://nests.tribal.gov.in/</t>
+          <t>https://www.emrs.tribal.gov.in/</t>
         </is>
       </c>
       <c r="G556" s="11" t="inlineStr">
@@ -16996,7 +16996,7 @@
       </c>
       <c r="I556" s="11" t="inlineStr">
         <is>
-          <t>EMRS recruitment is conducted by NESTS (own portal), not the Ministry homepage.</t>
+          <t>Dedicated EMRS recruitment/exam portal (apply/admit-card/results), distinct from NESTS org homepage.</t>
         </is>
       </c>
       <c r="J556" s="17" t="n">

</xml_diff>

<commit_message>
Batches 2 & 3/3: replace remaining homepage URLs with deep recruitment links
R557 NCST -> /recruitments-vacancies; R559 TRIFED -> /careers-list;
R561 EMRS -> emrs.tribal.gov.in portal; R571 NCPCR -> /index.php/recruitment;
R581 NYKS -> vacancies page; R593 CMTI -> /career/; R610 IITTM -> /Recruitment.html;
R584 LNIPE -> lnipe.in recruitment portal.
Flagged (SPA/unreachable, need manual deep-link): R33 PCI, R558 NSTFDC, R570 CARA, R586 NADA.
</commit_message>
<xml_diff>
--- a/Master list - Ministries and Departments.xlsx
+++ b/Master list - Ministries and Departments.xlsx
@@ -17030,12 +17030,12 @@
       </c>
       <c r="E557" s="11" t="inlineStr">
         <is>
-          <t>https://ncst.nic.in/</t>
+          <t>https://ncst.nic.in/recruitments-vacancies</t>
         </is>
       </c>
       <c r="F557" s="11" t="inlineStr">
         <is>
-          <t>https://ncst.nic.in/</t>
+          <t>https://ncst.nic.in/recruitments-vacancies</t>
         </is>
       </c>
       <c r="G557" s="11" t="inlineStr">
@@ -17045,12 +17045,12 @@
       </c>
       <c r="H557" s="11" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I557" s="11" t="inlineStr">
         <is>
-          <t>NCST publishes vacancies on its own official site.</t>
+          <t>NCST recruitments &amp; vacancies page (replaces homepage).</t>
         </is>
       </c>
       <c r="J557" s="17" t="n">
@@ -17099,12 +17099,12 @@
       </c>
       <c r="H558" s="11" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="I558" s="11" t="inlineStr">
         <is>
-          <t>NSTFDC official site; not reachable for deep-link confirmation from here.</t>
+          <t>NSTFDC site unreachable for deep-link confirmation from sandbox; recruitment notices are on the official site. NEEDS MANUAL CONFIRMATION.</t>
         </is>
       </c>
       <c r="J558" s="17" t="n">
@@ -17138,12 +17138,12 @@
       </c>
       <c r="E559" s="11" t="inlineStr">
         <is>
-          <t>https://trifed.tribal.gov.in/</t>
+          <t>https://trifed.tribal.gov.in/careers-list</t>
         </is>
       </c>
       <c r="F559" s="11" t="inlineStr">
         <is>
-          <t>https://trifed.tribal.gov.in/</t>
+          <t>https://trifed.tribal.gov.in/careers-list</t>
         </is>
       </c>
       <c r="G559" s="11" t="inlineStr">
@@ -17158,7 +17158,7 @@
       </c>
       <c r="I559" s="11" t="inlineStr">
         <is>
-          <t>TRIFED publishes its own recruitment (Careers) on its portal.</t>
+          <t>TRIFED careers list page (replaces homepage).</t>
         </is>
       </c>
       <c r="J559" s="17" t="n">
@@ -17246,12 +17246,12 @@
       </c>
       <c r="E561" s="11" t="inlineStr">
         <is>
-          <t>https://nests.tribal.gov.in/</t>
+          <t>https://www.emrs.tribal.gov.in/</t>
         </is>
       </c>
       <c r="F561" s="11" t="inlineStr">
         <is>
-          <t>https://nests.tribal.gov.in/</t>
+          <t>https://www.emrs.tribal.gov.in/</t>
         </is>
       </c>
       <c r="G561" s="11" t="inlineStr">
@@ -17266,7 +17266,7 @@
       </c>
       <c r="I561" s="11" t="inlineStr">
         <is>
-          <t>EMRS regional/field-unit recruitment via NESTS portal.</t>
+          <t>Dedicated EMRS recruitment/exam portal (apply/admit-card/results), distinct from NESTS org homepage.</t>
         </is>
       </c>
       <c r="J561" s="17" t="n">
@@ -17726,7 +17726,7 @@
       </c>
       <c r="I570" s="11" t="inlineStr">
         <is>
-          <t>CARA publishes recruitment on its own site; dedicated deep page not auto-confirmed.</t>
+          <t>CARA landing page surfaces current recruitment/deputation vacancy notices (PDFs); no separate recruitment route found. Flag for manual deep-link.</t>
         </is>
       </c>
       <c r="J570" s="17" t="n">
@@ -17760,12 +17760,12 @@
       </c>
       <c r="E571" s="11" t="inlineStr">
         <is>
-          <t>https://ncpcr.gov.in/</t>
+          <t>https://ncpcr.gov.in/index.php/recruitment</t>
         </is>
       </c>
       <c r="F571" s="11" t="inlineStr">
         <is>
-          <t>https://ncpcr.gov.in/</t>
+          <t>https://ncpcr.gov.in/index.php/recruitment</t>
         </is>
       </c>
       <c r="G571" s="11" t="inlineStr">
@@ -17775,12 +17775,12 @@
       </c>
       <c r="H571" s="11" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I571" s="11" t="inlineStr">
         <is>
-          <t>NCPCR publishes vacancies on its own official site.</t>
+          <t>NCPCR recruitment page (replaces homepage).</t>
         </is>
       </c>
       <c r="J571" s="17" t="n">
@@ -18274,12 +18274,12 @@
       </c>
       <c r="E581" s="11" t="inlineStr">
         <is>
-          <t>https://nyks.nic.in/</t>
+          <t>https://nyks.nic.in/resources/vacanciesNO.aspx</t>
         </is>
       </c>
       <c r="F581" s="11" t="inlineStr">
         <is>
-          <t>https://nyks.nic.in/</t>
+          <t>https://nyks.nic.in/resources/vacanciesNO.aspx</t>
         </is>
       </c>
       <c r="G581" s="11" t="inlineStr">
@@ -18289,12 +18289,12 @@
       </c>
       <c r="H581" s="11" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I581" s="11" t="inlineStr">
         <is>
-          <t>NYKS publishes recruitment on its own official site.</t>
+          <t>NYKS vacancies page (replaces homepage).</t>
         </is>
       </c>
       <c r="J581" s="17" t="n">
@@ -18436,12 +18436,12 @@
       </c>
       <c r="E584" s="11" t="inlineStr">
         <is>
-          <t>https://www.lnipe.gov.in/</t>
+          <t>https://www.lnipe.in/</t>
         </is>
       </c>
       <c r="F584" s="11" t="inlineStr">
         <is>
-          <t>https://www.lnipe.gov.in/</t>
+          <t>https://www.lnipe.in/</t>
         </is>
       </c>
       <c r="G584" s="11" t="inlineStr">
@@ -18456,7 +18456,7 @@
       </c>
       <c r="I584" s="11" t="inlineStr">
         <is>
-          <t>LNIPE official site; deep recruitment link not reachable for confirmation from here.</t>
+          <t>Dedicated LNIPE recruitment/online-application portal; main institute site is lnipe.gov.in.</t>
         </is>
       </c>
       <c r="J584" s="17" t="n">
@@ -18464,7 +18464,7 @@
       </c>
       <c r="K584" s="11" t="inlineStr">
         <is>
-          <t>Website</t>
+          <t>Portal</t>
         </is>
       </c>
     </row>
@@ -18559,12 +18559,12 @@
       </c>
       <c r="H586" s="11" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="I586" s="11" t="inlineStr">
         <is>
-          <t>NADA India official portal.</t>
+          <t>NADA recruitment posted on its official site (apply online via nadaindia.yas.gov.in); SPA prevented deep-link confirmation. Flag for manual deep-link.</t>
         </is>
       </c>
       <c r="J586" s="17" t="n">
@@ -18572,7 +18572,7 @@
       </c>
       <c r="K586" s="11" t="inlineStr">
         <is>
-          <t>Portal</t>
+          <t>Website</t>
         </is>
       </c>
     </row>
@@ -18896,12 +18896,12 @@
       </c>
       <c r="E593" s="11" t="inlineStr">
         <is>
-          <t>https://cmti.res.in/</t>
+          <t>https://cmti.res.in/career/</t>
         </is>
       </c>
       <c r="F593" s="11" t="inlineStr">
         <is>
-          <t>https://cmti.res.in/</t>
+          <t>https://cmti.res.in/career/</t>
         </is>
       </c>
       <c r="G593" s="11" t="inlineStr">
@@ -18911,12 +18911,12 @@
       </c>
       <c r="H593" s="11" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I593" s="11" t="inlineStr">
         <is>
-          <t>CMTI official site; careers page not reachable for confirmation from here.</t>
+          <t>CMTI Careers page (replaces homepage); active walk-in recruitment notices listed.</t>
         </is>
       </c>
       <c r="J593" s="17" t="n">
@@ -19762,12 +19762,12 @@
       </c>
       <c r="E610" s="11" t="inlineStr">
         <is>
-          <t>https://www.iittm.ac.in/</t>
+          <t>https://www.iittm.ac.in/Recruitment.html</t>
         </is>
       </c>
       <c r="F610" s="11" t="inlineStr">
         <is>
-          <t>https://www.iittm.ac.in/</t>
+          <t>https://www.iittm.ac.in/Recruitment.html</t>
         </is>
       </c>
       <c r="G610" s="11" t="inlineStr">
@@ -19777,12 +19777,12 @@
       </c>
       <c r="H610" s="11" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="I610" s="11" t="inlineStr">
         <is>
-          <t>IITTM posts vacancy advertisements as notifications on its site; Director-level posts also via Ministry of Tourism recruitment page.</t>
+          <t>IITTM recruitment page (replaces homepage); Director-level posts also advertised via tourism.gov.in/recruitment.</t>
         </is>
       </c>
       <c r="J610" s="17" t="n">

</xml_diff>

<commit_message>
Second pass on 4 flagged rows: resolve CARA + NADA; PCI + NSTFDC still need manual check
R570 CARA -> /resource/Archive.html (recruitment listing, confirmed live)
R586 NADA -> /career-opportunities/ (per official site nav; domain network-blocked from sandbox)
R33 PCI, R558 NSTFDC -> remain flagged Low (SPA / unreachable; no recruitment route found)
</commit_message>
<xml_diff>
--- a/Master list - Ministries and Departments.xlsx
+++ b/Master list - Ministries and Departments.xlsx
@@ -2105,7 +2105,7 @@
       </c>
       <c r="I33" s="11" t="inlineStr">
         <is>
-          <t>Domain corrected pci.nic.in -&gt; pci.gov.in. Site is a SPA exposing no stable recruitment-route URL; vacancy notices appear within portal. NEEDS MANUAL CONFIRMATION.</t>
+          <t>Second pass: no stable recruitment-route URL found (pci.gov.in is a SPA; old pci.nic.in unreachable). Recruitment notices appear within the portal. STILL NEEDS MANUAL CONFIRMATION.</t>
         </is>
       </c>
       <c r="J33" s="17" t="n">
@@ -17104,7 +17104,7 @@
       </c>
       <c r="I558" s="11" t="inlineStr">
         <is>
-          <t>NSTFDC site unreachable for deep-link confirmation from sandbox; recruitment notices are on the official site. NEEDS MANUAL CONFIRMATION.</t>
+          <t>Second pass: nstfdc.in unreachable from sandbox and not indexed for a recruitment route. Recruitment notices are on the official site. STILL NEEDS MANUAL CONFIRMATION.</t>
         </is>
       </c>
       <c r="J558" s="17" t="n">
@@ -17706,12 +17706,12 @@
       </c>
       <c r="E570" s="11" t="inlineStr">
         <is>
-          <t>https://cara.wcd.gov.in/</t>
+          <t>https://cara.wcd.gov.in/resource/Archive.html</t>
         </is>
       </c>
       <c r="F570" s="11" t="inlineStr">
         <is>
-          <t>https://cara.wcd.gov.in/</t>
+          <t>https://cara.wcd.gov.in/resource/Archive.html</t>
         </is>
       </c>
       <c r="G570" s="11" t="inlineStr">
@@ -17726,7 +17726,7 @@
       </c>
       <c r="I570" s="11" t="inlineStr">
         <is>
-          <t>CARA landing page surfaces current recruitment/deputation vacancy notices (PDFs); no separate recruitment route found. Flag for manual deep-link.</t>
+          <t>CARA recruitment listing page (posts open for application); replaces homepage. Confirmed live.</t>
         </is>
       </c>
       <c r="J570" s="17" t="n">
@@ -18544,12 +18544,12 @@
       </c>
       <c r="E586" s="11" t="inlineStr">
         <is>
-          <t>https://nadaindia.yas.gov.in/</t>
+          <t>https://nadaindia.yas.gov.in/career-opportunities/</t>
         </is>
       </c>
       <c r="F586" s="11" t="inlineStr">
         <is>
-          <t>https://nadaindia.yas.gov.in/</t>
+          <t>https://nadaindia.yas.gov.in/career-opportunities/</t>
         </is>
       </c>
       <c r="G586" s="11" t="inlineStr">
@@ -18564,7 +18564,7 @@
       </c>
       <c r="I586" s="11" t="inlineStr">
         <is>
-          <t>NADA recruitment posted on its official site (apply online via nadaindia.yas.gov.in); SPA prevented deep-link confirmation. Flag for manual deep-link.</t>
+          <t>NADA 'Career Opportunities' page (per official site navigation). Domain network-blocked from sandbox, so slug is evidence-based, not curl-verified.</t>
         </is>
       </c>
       <c r="J586" s="17" t="n">

</xml_diff>

<commit_message>
Next set batch: fill NIPER + Civil Aviation + Coal clusters (15 orgs)
Civil Aviation (R35,R37-44): MoCA aviation-jobs, DGCA recruitment, AAI careers,
IGRUA/RGNAU careers, NIPER jobs; AAIB & BCAS flagged (SPA/no route).
Coal (R46-51): MoC advertisements, CCO recruitment, CIL careers, SCCL careers.
- SCCL has a SEPARATE deputation page (careersDep.asp) -> G=No, F set distinctly.
- NIMH merged into NIOH (ICMR, 2019) -> points to NIOH recruitments.
Bare 'Ministry of X' parent rows left blank per convention.
</commit_message>
<xml_diff>
--- a/Master list - Ministries and Departments.xlsx
+++ b/Master list - Ministries and Departments.xlsx
@@ -17,9 +17,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="dd-mm-yyyy"/>
+    <numFmt numFmtId="166" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -2191,13 +2192,39 @@
           <t>Autonomous Body</t>
         </is>
       </c>
-      <c r="E35" s="11" t="n"/>
-      <c r="F35" s="11" t="n"/>
-      <c r="G35" s="11" t="n"/>
-      <c r="H35" s="11" t="n"/>
-      <c r="I35" s="11" t="n"/>
-      <c r="J35" s="11" t="n"/>
-      <c r="K35" s="11" t="n"/>
+      <c r="E35" s="11" t="inlineStr">
+        <is>
+          <t>https://www.niper.gov.in/jobs</t>
+        </is>
+      </c>
+      <c r="F35" s="11" t="inlineStr">
+        <is>
+          <t>https://www.niper.gov.in/jobs</t>
+        </is>
+      </c>
+      <c r="G35" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H35" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I35" s="11" t="inlineStr">
+        <is>
+          <t>NIPER jobs page (NIPER Mohali; sister NIPER campuses recruit on their own institute sites).</t>
+        </is>
+      </c>
+      <c r="J35" s="17" t="n">
+        <v>46183</v>
+      </c>
+      <c r="K35" s="11" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
     </row>
     <row r="36" ht="15.75" customHeight="1" s="16">
       <c r="A36" s="4">
@@ -2247,13 +2274,39 @@
           <t>Attached Office</t>
         </is>
       </c>
-      <c r="E37" s="11" t="n"/>
-      <c r="F37" s="11" t="n"/>
-      <c r="G37" s="11" t="n"/>
-      <c r="H37" s="11" t="n"/>
-      <c r="I37" s="11" t="n"/>
-      <c r="J37" s="11" t="n"/>
-      <c r="K37" s="11" t="n"/>
+      <c r="E37" s="11" t="inlineStr">
+        <is>
+          <t>https://www.civilaviation.gov.in/aviation-jobs</t>
+        </is>
+      </c>
+      <c r="F37" s="11" t="inlineStr">
+        <is>
+          <t>https://www.civilaviation.gov.in/aviation-jobs</t>
+        </is>
+      </c>
+      <c r="G37" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H37" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I37" s="11" t="inlineStr">
+        <is>
+          <t>Ministry of Civil Aviation 'Aviation Jobs' page.</t>
+        </is>
+      </c>
+      <c r="J37" s="17" t="n">
+        <v>46183</v>
+      </c>
+      <c r="K37" s="11" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="15.75" customHeight="1" s="16">
       <c r="A38" s="4">
@@ -2275,13 +2328,39 @@
           <t>Attached Office</t>
         </is>
       </c>
-      <c r="E38" s="11" t="n"/>
-      <c r="F38" s="11" t="n"/>
-      <c r="G38" s="11" t="n"/>
-      <c r="H38" s="11" t="n"/>
-      <c r="I38" s="11" t="n"/>
-      <c r="J38" s="11" t="n"/>
-      <c r="K38" s="11" t="n"/>
+      <c r="E38" s="11" t="inlineStr">
+        <is>
+          <t>https://www.dgca.gov.in/digigov-portal/?page=jsp/dgca/homePage/instructions/RECRUITMENT.html</t>
+        </is>
+      </c>
+      <c r="F38" s="11" t="inlineStr">
+        <is>
+          <t>https://www.dgca.gov.in/digigov-portal/?page=jsp/dgca/homePage/instructions/RECRUITMENT.html</t>
+        </is>
+      </c>
+      <c r="G38" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H38" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I38" s="11" t="inlineStr">
+        <is>
+          <t>DGCA recruitment page.</t>
+        </is>
+      </c>
+      <c r="J38" s="17" t="n">
+        <v>46183</v>
+      </c>
+      <c r="K38" s="11" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="15.75" customHeight="1" s="16">
       <c r="A39" s="4">
@@ -2303,13 +2382,39 @@
           <t>Attached Office</t>
         </is>
       </c>
-      <c r="E39" s="11" t="n"/>
-      <c r="F39" s="11" t="n"/>
-      <c r="G39" s="11" t="n"/>
-      <c r="H39" s="11" t="n"/>
-      <c r="I39" s="11" t="n"/>
-      <c r="J39" s="11" t="n"/>
-      <c r="K39" s="11" t="n"/>
+      <c r="E39" s="11" t="inlineStr">
+        <is>
+          <t>https://www.civilaviation.gov.in/aviation-jobs</t>
+        </is>
+      </c>
+      <c r="F39" s="11" t="inlineStr">
+        <is>
+          <t>https://www.civilaviation.gov.in/aviation-jobs</t>
+        </is>
+      </c>
+      <c r="G39" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H39" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I39" s="11" t="inlineStr">
+        <is>
+          <t>BCAS vacancies aggregated on MoCA Aviation Jobs page; BCAS recruits largely by deputation. Own site bcasindia.gov.in is a SPA with no dedicated recruitment route.</t>
+        </is>
+      </c>
+      <c r="J39" s="17" t="n">
+        <v>46183</v>
+      </c>
+      <c r="K39" s="11" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="15.75" customHeight="1" s="16">
       <c r="A40" s="4">
@@ -2331,13 +2436,39 @@
           <t>Attached Office</t>
         </is>
       </c>
-      <c r="E40" s="11" t="n"/>
-      <c r="F40" s="11" t="n"/>
-      <c r="G40" s="11" t="n"/>
-      <c r="H40" s="11" t="n"/>
-      <c r="I40" s="11" t="n"/>
-      <c r="J40" s="11" t="n"/>
-      <c r="K40" s="11" t="n"/>
+      <c r="E40" s="11" t="inlineStr">
+        <is>
+          <t>https://aaib.gov.in/</t>
+        </is>
+      </c>
+      <c r="F40" s="11" t="inlineStr">
+        <is>
+          <t>https://aaib.gov.in/</t>
+        </is>
+      </c>
+      <c r="G40" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H40" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I40" s="11" t="inlineStr">
+        <is>
+          <t>AAIB posts vacancy circulars on its homepage (What's New); no dedicated recruitment route found. Flag for manual deep-link.</t>
+        </is>
+      </c>
+      <c r="J40" s="17" t="n">
+        <v>46183</v>
+      </c>
+      <c r="K40" s="11" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="15.75" customHeight="1" s="16">
       <c r="A41" s="4">
@@ -2359,13 +2490,39 @@
           <t>Statutory Body</t>
         </is>
       </c>
-      <c r="E41" s="11" t="n"/>
-      <c r="F41" s="11" t="n"/>
-      <c r="G41" s="11" t="n"/>
-      <c r="H41" s="11" t="n"/>
-      <c r="I41" s="11" t="n"/>
-      <c r="J41" s="11" t="n"/>
-      <c r="K41" s="11" t="n"/>
+      <c r="E41" s="11" t="inlineStr">
+        <is>
+          <t>https://www.aai.aero/en/careers</t>
+        </is>
+      </c>
+      <c r="F41" s="11" t="inlineStr">
+        <is>
+          <t>https://www.aai.aero/en/careers</t>
+        </is>
+      </c>
+      <c r="G41" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H41" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I41" s="11" t="inlineStr">
+        <is>
+          <t>Airports Authority of India careers section.</t>
+        </is>
+      </c>
+      <c r="J41" s="17" t="n">
+        <v>46183</v>
+      </c>
+      <c r="K41" s="11" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="15.75" customHeight="1" s="16">
       <c r="A42" s="4">
@@ -2387,13 +2544,39 @@
           <t>Autonomous Body</t>
         </is>
       </c>
-      <c r="E42" s="11" t="n"/>
-      <c r="F42" s="11" t="n"/>
-      <c r="G42" s="11" t="n"/>
-      <c r="H42" s="11" t="n"/>
-      <c r="I42" s="11" t="n"/>
-      <c r="J42" s="11" t="n"/>
-      <c r="K42" s="11" t="n"/>
+      <c r="E42" s="11" t="inlineStr">
+        <is>
+          <t>https://www.igrua.gov.in/careers</t>
+        </is>
+      </c>
+      <c r="F42" s="11" t="inlineStr">
+        <is>
+          <t>https://www.igrua.gov.in/careers</t>
+        </is>
+      </c>
+      <c r="G42" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H42" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I42" s="11" t="inlineStr">
+        <is>
+          <t>IGRUA careers page.</t>
+        </is>
+      </c>
+      <c r="J42" s="17" t="n">
+        <v>46183</v>
+      </c>
+      <c r="K42" s="11" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="15.75" customHeight="1" s="16">
       <c r="A43" s="4">
@@ -2415,13 +2598,39 @@
           <t>Autonomous Body</t>
         </is>
       </c>
-      <c r="E43" s="11" t="n"/>
-      <c r="F43" s="11" t="n"/>
-      <c r="G43" s="11" t="n"/>
-      <c r="H43" s="11" t="n"/>
-      <c r="I43" s="11" t="n"/>
-      <c r="J43" s="11" t="n"/>
-      <c r="K43" s="11" t="n"/>
+      <c r="E43" s="11" t="inlineStr">
+        <is>
+          <t>https://www.rgnau.ac.in/en/careers.html</t>
+        </is>
+      </c>
+      <c r="F43" s="11" t="inlineStr">
+        <is>
+          <t>https://www.rgnau.ac.in/en/careers.html</t>
+        </is>
+      </c>
+      <c r="G43" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H43" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I43" s="11" t="inlineStr">
+        <is>
+          <t>RGNAU careers page.</t>
+        </is>
+      </c>
+      <c r="J43" s="17" t="n">
+        <v>46183</v>
+      </c>
+      <c r="K43" s="11" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="15.75" customHeight="1" s="16">
       <c r="A44" s="4">
@@ -2443,13 +2652,39 @@
           <t>Subordinate Office</t>
         </is>
       </c>
-      <c r="E44" s="11" t="n"/>
-      <c r="F44" s="11" t="n"/>
-      <c r="G44" s="11" t="n"/>
-      <c r="H44" s="11" t="n"/>
-      <c r="I44" s="11" t="n"/>
-      <c r="J44" s="11" t="n"/>
-      <c r="K44" s="11" t="n"/>
+      <c r="E44" s="11" t="inlineStr">
+        <is>
+          <t>https://www.dgca.gov.in/digigov-portal/?page=jsp/dgca/homePage/instructions/RECRUITMENT.html</t>
+        </is>
+      </c>
+      <c r="F44" s="11" t="inlineStr">
+        <is>
+          <t>https://www.dgca.gov.in/digigov-portal/?page=jsp/dgca/homePage/instructions/RECRUITMENT.html</t>
+        </is>
+      </c>
+      <c r="G44" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H44" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I44" s="11" t="inlineStr">
+        <is>
+          <t>DGCA Regional Airworthiness field units; recruitment via DGCA recruitment page.</t>
+        </is>
+      </c>
+      <c r="J44" s="17" t="n">
+        <v>46183</v>
+      </c>
+      <c r="K44" s="11" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="15.75" customHeight="1" s="16">
       <c r="A45" s="4">
@@ -2499,13 +2734,39 @@
           <t>Attached Office</t>
         </is>
       </c>
-      <c r="E46" s="11" t="n"/>
-      <c r="F46" s="11" t="n"/>
-      <c r="G46" s="11" t="n"/>
-      <c r="H46" s="11" t="n"/>
-      <c r="I46" s="11" t="n"/>
-      <c r="J46" s="11" t="n"/>
-      <c r="K46" s="11" t="n"/>
+      <c r="E46" s="11" t="inlineStr">
+        <is>
+          <t>https://coal.gov.in/public-information/advertisements</t>
+        </is>
+      </c>
+      <c r="F46" s="11" t="inlineStr">
+        <is>
+          <t>https://coal.gov.in/public-information/advertisements</t>
+        </is>
+      </c>
+      <c r="G46" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H46" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I46" s="11" t="inlineStr">
+        <is>
+          <t>Ministry of Coal advertisements (incl. recruitment/vacancy circulars).</t>
+        </is>
+      </c>
+      <c r="J46" s="17" t="n">
+        <v>46183</v>
+      </c>
+      <c r="K46" s="11" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="15.75" customHeight="1" s="16">
       <c r="A47" s="4">
@@ -2527,13 +2788,39 @@
           <t>Attached Office</t>
         </is>
       </c>
-      <c r="E47" s="11" t="n"/>
-      <c r="F47" s="11" t="n"/>
-      <c r="G47" s="11" t="n"/>
-      <c r="H47" s="11" t="n"/>
-      <c r="I47" s="11" t="n"/>
-      <c r="J47" s="11" t="n"/>
-      <c r="K47" s="11" t="n"/>
+      <c r="E47" s="11" t="inlineStr">
+        <is>
+          <t>https://www.coalcontroller.gov.in/recruitment</t>
+        </is>
+      </c>
+      <c r="F47" s="11" t="inlineStr">
+        <is>
+          <t>https://www.coalcontroller.gov.in/recruitment</t>
+        </is>
+      </c>
+      <c r="G47" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H47" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I47" s="11" t="inlineStr">
+        <is>
+          <t>Coal Controller Organisation recruitment page.</t>
+        </is>
+      </c>
+      <c r="J47" s="17" t="n">
+        <v>46183</v>
+      </c>
+      <c r="K47" s="11" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="15.75" customHeight="1" s="16">
       <c r="A48" s="4">
@@ -2555,13 +2842,39 @@
           <t>Subordinate Office</t>
         </is>
       </c>
-      <c r="E48" s="11" t="n"/>
-      <c r="F48" s="11" t="n"/>
-      <c r="G48" s="11" t="n"/>
-      <c r="H48" s="11" t="n"/>
-      <c r="I48" s="11" t="n"/>
-      <c r="J48" s="11" t="n"/>
-      <c r="K48" s="11" t="n"/>
+      <c r="E48" s="11" t="inlineStr">
+        <is>
+          <t>https://www.coalcontroller.gov.in/recruitment</t>
+        </is>
+      </c>
+      <c r="F48" s="11" t="inlineStr">
+        <is>
+          <t>https://www.coalcontroller.gov.in/recruitment</t>
+        </is>
+      </c>
+      <c r="G48" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H48" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I48" s="11" t="inlineStr">
+        <is>
+          <t>Coal Controller's field offices; recruitment via Coal Controller Organisation.</t>
+        </is>
+      </c>
+      <c r="J48" s="17" t="n">
+        <v>46183</v>
+      </c>
+      <c r="K48" s="11" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="15.75" customHeight="1" s="16">
       <c r="A49" s="4">
@@ -2583,13 +2896,39 @@
           <t>Autonomous Body</t>
         </is>
       </c>
-      <c r="E49" s="11" t="n"/>
-      <c r="F49" s="11" t="n"/>
-      <c r="G49" s="11" t="n"/>
-      <c r="H49" s="11" t="n"/>
-      <c r="I49" s="11" t="n"/>
-      <c r="J49" s="11" t="n"/>
-      <c r="K49" s="11" t="n"/>
+      <c r="E49" s="11" t="inlineStr">
+        <is>
+          <t>https://nioh.org/recruitments/</t>
+        </is>
+      </c>
+      <c r="F49" s="11" t="inlineStr">
+        <is>
+          <t>https://nioh.org/recruitments/</t>
+        </is>
+      </c>
+      <c r="G49" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H49" s="11" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="I49" s="11" t="inlineStr">
+        <is>
+          <t>NIMH merged with NIOH (ICMR) in 2019; recruitment via NIOH recruitments page.</t>
+        </is>
+      </c>
+      <c r="J49" s="17" t="n">
+        <v>46183</v>
+      </c>
+      <c r="K49" s="11" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="15.75" customHeight="1" s="16">
       <c r="A50" s="4">
@@ -2611,13 +2950,39 @@
           <t>PSU / Board / Trust</t>
         </is>
       </c>
-      <c r="E50" s="11" t="n"/>
-      <c r="F50" s="11" t="n"/>
-      <c r="G50" s="11" t="n"/>
-      <c r="H50" s="11" t="n"/>
-      <c r="I50" s="11" t="n"/>
-      <c r="J50" s="11" t="n"/>
-      <c r="K50" s="11" t="n"/>
+      <c r="E50" s="11" t="inlineStr">
+        <is>
+          <t>https://www.coalindia.in/career-cil/</t>
+        </is>
+      </c>
+      <c r="F50" s="11" t="inlineStr">
+        <is>
+          <t>https://www.coalindia.in/career-cil/</t>
+        </is>
+      </c>
+      <c r="G50" s="11" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="H50" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I50" s="11" t="inlineStr">
+        <is>
+          <t>Coal India Limited careers page.</t>
+        </is>
+      </c>
+      <c r="J50" s="17" t="n">
+        <v>46183</v>
+      </c>
+      <c r="K50" s="11" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="15.75" customHeight="1" s="16">
       <c r="A51" s="4">
@@ -2639,13 +3004,39 @@
           <t>PSU / Board / Trust</t>
         </is>
       </c>
-      <c r="E51" s="11" t="n"/>
-      <c r="F51" s="11" t="n"/>
-      <c r="G51" s="11" t="n"/>
-      <c r="H51" s="11" t="n"/>
-      <c r="I51" s="11" t="n"/>
-      <c r="J51" s="11" t="n"/>
-      <c r="K51" s="11" t="n"/>
+      <c r="E51" s="11" t="inlineStr">
+        <is>
+          <t>https://www.scclmines.com/scclnew/careers.asp</t>
+        </is>
+      </c>
+      <c r="F51" s="11" t="inlineStr">
+        <is>
+          <t>https://www.scclmines.com/scclnew/careersDep.asp</t>
+        </is>
+      </c>
+      <c r="G51" s="11" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H51" s="11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="I51" s="11" t="inlineStr">
+        <is>
+          <t>SCCL careers page; deputation vacancies are on a SEPARATE page (careersDep.asp).</t>
+        </is>
+      </c>
+      <c r="J51" s="17" t="n">
+        <v>46183</v>
+      </c>
+      <c r="K51" s="11" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="15.75" customHeight="1" s="16">
       <c r="A52" s="4">

</xml_diff>